<commit_message>
Fix critical issues from code review before ordering
1. CRITICAL: Replace 100µF cap with 220µF (GRM31CR60J227ME11L)
   - X5R ceramic derates ~35% at 3V DC bias: 100µF → ~65µF (below 120µF needed)
   - 220µF → ~143µF effective. Safely exceeds 120µF TX burst requirement.
   - Same 1206 package, same 1.6mm height. $0.20/ea.

2. CRITICAL: Delete stale BOM.md (still referenced obsolete Honeywell ABP)
   - Excel BOM is now the single source of truth

3. IMPORTANT: Mark 100Ω resistors as SPARE in BOM notes
   - Series R with ceramic buffer cap creates 1.2V drop at 12mA — defeats purpose
   - Keep parts but do NOT place in series with TX buffer cap

4. IMPORTANT: Document MS5837-30BA -20°C limitation in spec
   - Sensor rated -20 to +85°C, our spec says -30°C
   - Sensor will function but accuracy not guaranteed below -20°C
   - Acceptable for v1, test during prototyping

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -107,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -129,11 +129,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,6 +211,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,6 +605,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -607,13 +654,6 @@
           <t>ELECTRONICS</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="50" customHeight="1">
       <c r="A6" s="6" t="n">
@@ -735,12 +775,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>TX Buffer Capacitor (100µF)</t>
+          <t>TX Buffer Capacitor (220µF)</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>GRM31CR60J107ME39L</t>
+          <t>GRM31CR60J227ME11L</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -753,17 +793,17 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>$0.15</t>
+          <t>$0.20</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>$0.45</t>
+          <t>$0.60</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Murata 100µF 6.3V X5R 1206 ceramic. Replaces supercap — only 120µF needed for TX burst buffer. 1.6mm tall. Millions in stock.</t>
+          <t>Murata 220µF 6.3V X5R 1206 ceramic. After ~35% DC bias derating at 3V → ~143µF effective. Exceeds 120µF requirement. 1.6mm tall. Replaces 100µF (which derated to ~65µF — insufficient).</t>
         </is>
       </c>
     </row>
@@ -915,7 +955,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Yageo 1%. Supercap charge-limit (now buffer cap series R). 3.7M in stock.</t>
+          <t>Yageo 1%. SPARE PARTS — do NOT place in series with TX buffer cap. Original supercap charge-limit purpose no longer applies. Use for other circuit needs or keep as spares.</t>
         </is>
       </c>
     </row>
@@ -925,13 +965,6 @@
           <t>DEV TOOLS (one-time)</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
     </row>
     <row r="15" ht="50" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -1015,18 +1048,19 @@
           <t>DigiKey Order Total</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="22" t="n"/>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>~$282.61</t>
+          <t>~$282.76</t>
         </is>
       </c>
       <c r="H17" s="9" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19" ht="35" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
@@ -1116,11 +1150,6 @@
           <t>BATTERIES</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="7" t="n">
@@ -1158,11 +1187,6 @@
           <t>MECHANICAL</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -1290,11 +1314,6 @@
           <t>CONSUMABLES</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -1422,11 +1441,6 @@
           <t>PCB FABRICATION</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="7" t="n">
@@ -1464,9 +1478,9 @@
           <t>Amazon/Other Total</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
       <c r="E19" s="10" t="inlineStr">
         <is>
           <t>~$75-104</t>
@@ -1492,8 +1506,8 @@
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A19:D19"/>
@@ -1539,9 +1553,6 @@
           <t>ORDER NOW — Need for firmware dev</t>
         </is>
       </c>
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1637,9 +1648,6 @@
           <t>ORDER AFTER KICAD DONE</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -1669,9 +1677,6 @@
           <t>ORDER ANYTIME</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1841,6 +1846,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
@@ -1972,7 +1978,7 @@
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>GRM31CR60J107ME39L</t>
+          <t>GRM31CR60J227ME11L</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
@@ -2065,6 +2071,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add complete project documentation, Gerber files, and GitHub structure
- README with full project description, specs, BOM, and build instructions
- CERN OHL v2 (hardware) and MIT (software) licenses
- Design spec Rev 8 and implementation plan Rev 8
- PCB Gerber files v23 ready for fabrication (16x42mm, 2-layer, ENIG)
- BOM spreadsheet with DigiKey/Mouser/Amazon/AliExpress sourcing
- Competitive comparison vs SRAM TyreWiz 2.0
- Fusion 360 schematic guide
- PCBWay sponsorship acknowledgment

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DigiKey Order" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -29,38 +28,48 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="FF666666"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00238636"/>
+      <color rgb="FF238636"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00CC6600"/>
+      <color rgb="FFCC6600"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="8">
@@ -72,38 +81,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
-        <bgColor rgb="002F5496"/>
+        <fgColor rgb="FF2F5496"/>
+        <bgColor rgb="FF2F5496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4EC"/>
-        <bgColor rgb="00FCE4EC"/>
+        <fgColor rgb="FFFCE4EC"/>
+        <bgColor rgb="FFFCE4EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
-        <bgColor rgb="00E8F5E9"/>
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3E0"/>
-        <bgColor rgb="00FFF3E0"/>
+        <fgColor rgb="FFFFF3E0"/>
+        <bgColor rgb="FFFFF3E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,23 +126,48 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -141,81 +175,56 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -579,505 +588,491 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" style="11" min="1" max="1"/>
+    <col width="30" customWidth="1" style="11" min="2" max="2"/>
+    <col width="28" customWidth="1" style="11" min="3" max="3"/>
+    <col width="10" customWidth="1" style="11" min="4" max="4"/>
+    <col width="8" customWidth="1" style="11" min="5" max="5"/>
+    <col width="12" customWidth="1" style="11" min="6" max="6"/>
+    <col width="14" customWidth="1" style="11" min="7" max="7"/>
+    <col width="55" customWidth="1" style="11" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>OpenTPMS — DigiKey Order (3 sensors: 1 pair + 1 spare)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Updated 2026-04-02. All parts verified against design spec + datasheets.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>DigiKey Part Number</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>ELECTRONICS</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="6" t="n">
+    <row r="6" ht="50" customHeight="1" s="11">
+      <c r="A6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>nRF52 BLE+ANT+ Module</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>MDBT42Q-512KV2</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>$4.95</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>$14.85</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Raytac. 1.7-3.6V. Marketplace item — may need manual search. Backup: LCSC $5.96.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="6" t="n">
+    <row r="7" ht="50" customHeight="1" s="11">
+      <c r="A7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Pressure Sensor (30bar abs)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>MS583730BA01-50</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>$11.09</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>$33.27</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>TE MS5837-30BA. 1.5-3.6V. I2C 0x76. 3.3x3.3x2.75mm. Gel-filled. 6400+ in stock.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="7" t="n">
+    <row r="8" ht="50" customHeight="1" s="11">
+      <c r="A8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>3-Axis Accelerometer</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>LIS2DH12TR</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>$2.47</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>$7.41</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>ST Micro. 1.71-3.6V. I2C 0x19. 2x2x1mm. Motion-detect interrupt. 77k in stock.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="7" t="n">
+    <row r="9" ht="50" customHeight="1" s="11">
+      <c r="A9" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>TX Buffer Capacitor (220µF)</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>GRM31CR60J227ME11L</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>$0.20</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>$0.60</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Murata 220µF 6.3V X5R 1206 ceramic. After ~35% DC bias derating at 3V → ~143µF effective. Exceeds 120µF requirement. 1.6mm tall. Replaces 100µF (which derated to ~65µF — insufficient).</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="7" t="n">
+    <row r="10" ht="50" customHeight="1" s="11">
+      <c r="A10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>CR1225 Battery Holder SMD</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>BHSD-1225-SM</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>CR1225 Battery Contact</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Custom PCB pad + lid spring</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>No commercial holder. ~10mm ENIG pad on PCB (negative) + BeCu leaf spring in lid (positive). BeCu sheet from Amazon/AliExpress ~$3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1" s="11">
+      <c r="A11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>100nF Caps (0402 SMD)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>CL05B104KO5NNNC</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>$2.21</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>$6.63</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>MPD. 12mm coin cell SMD. 5.8k in stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="50" customHeight="1">
-      <c r="A11" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>100nF Caps (0402 SMD)</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>CL05B104KO5NNNC</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="E11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>$0.025</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>$0.50</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Samsung MLCC 16V X7R. Decoupling. 13M in stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1" s="11">
+      <c r="A12" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>4.7kΩ Resistors (0402)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>RC0402FR-074K7L</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>$0.025</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>$0.50</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Samsung MLCC 16V X7R. Decoupling. 13M in stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="50" customHeight="1">
-      <c r="A12" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>4.7kΩ Resistors (0402)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>RC0402FR-074K7L</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>$0.006</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>$0.06</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Yageo 1%. I2C pull-ups. 150 min qty on Mouser. ALSO ORDER: 6x 150pF 0402 NFC tuning caps + 3x 10uH 0402 inductors (DC-DC). Add to Mouser order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1" s="11">
+      <c r="A13" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>100Ω Resistors (0402)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>RC0402FR-07100RL</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E13" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>$0.006</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>$0.06</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Yageo 1%. I2C pull-ups. 3M in stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="50" customHeight="1">
-      <c r="A13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>100Ω Resistors (0402)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>RC0402FR-07100RL</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Yageo 1%. SPARE PARTS — do NOT place in series with TX buffer cap. Original supercap charge-limit purpose no longer applies. Use for other circuit needs or keep as spares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>DEV TOOLS (one-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1" s="11">
+      <c r="A15" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>nRF52-DK Dev Board</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>NRF52-DK</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>$52.77</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>$52.77</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Nordic. Built-in J-Link. Firmware dev before PCBs arrive. 656 in stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1" s="11">
+      <c r="A16" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>$0.006</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>$0.06</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>Yageo 1%. SPARE PARTS — do NOT place in series with TX buffer cap. Original supercap charge-limit purpose no longer applies. Use for other circuit needs or keep as spares.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>DEV TOOLS (one-time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="50" customHeight="1">
-      <c r="A15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>nRF52-DK Dev Board</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>NRF52-DK</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Power Profiler Kit II</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>NRF-PPK2</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>$52.77</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>$52.77</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>Nordic. Built-in J-Link. Firmware dev before PCBs arrive. 656 in stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="50" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Power Profiler Kit II</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>NRF-PPK2</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>$166.61</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>$166.61</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Nordic. nA-level current measurement. 561 in stock.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>DigiKey Order Total</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="22" t="n"/>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>~$282.76</t>
         </is>
       </c>
-      <c r="H17" s="9" t="n"/>
-    </row>
-    <row r="18"/>
-    <row r="19" ht="35" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="H17" s="4" t="n"/>
+    </row>
+    <row r="19" ht="35" customHeight="1" s="11">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>VERIFIED: All voltages compatible with CR1225 (3.0V). No I2C address conflicts (0x76 + 0x19). All components fit enclosure height budget (≤3.0mm). All in stock.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A5:H5"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -1088,433 +1083,420 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" style="11" min="1" max="1"/>
+    <col width="28" customWidth="1" style="11" min="2" max="2"/>
+    <col width="32" customWidth="1" style="11" min="3" max="3"/>
+    <col width="18" customWidth="1" style="11" min="4" max="4"/>
+    <col width="12" customWidth="1" style="11" min="5" max="5"/>
+    <col width="55" customWidth="1" style="11" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="19" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>OpenTPMS — Amazon / AliExpress / JLCPCB</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Items not on DigiKey</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Est. Price</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>BATTERIES</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="7" t="n">
+    <row r="6" ht="40" customHeight="1" s="11">
+      <c r="A6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>CR1225 Coin Cell</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Panasonic CR1225 x5</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>$3-5</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>3 installed + 2 spares</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>MECHANICAL</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="7" t="n">
+    <row r="8" ht="40" customHeight="1" s="11">
+      <c r="A8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>M1.2x3mm Allen Screws</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Stainless hex socket assortment</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>M1.4x3mm Allen Screws (DIN912)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Stainless hex socket cap screw (DIN912), 2.6mm head dia</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>C$2.46</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>50pcs M1.4 DIN912 304SS 3mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1" s="11">
+      <c r="A9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>M1.4 Heat-Set Inserts</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Brass knurled threaded, OD2.3mm, ~5.5mm boss dia required</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>C$3.70</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>100pcs M1.4 OD2.3mm brass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1" s="11">
+      <c r="A10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Silicone O-Rings</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>~12mm OD x 1mm silicone assortment</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>~$8-12</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Kit has 50+, need 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>M1.2 Heat-Set Inserts</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Brass knurled threaded assortment</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>~$5-8</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SILICONE not nitrile</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1" s="11">
+      <c r="A11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>ePTFE Vent Membrane</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>IP67 adhesive breathable discs</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>~$5-15</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Search "ePTFE waterproof vent adhesive"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>CONSUMABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1" s="11">
+      <c r="A13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Conformal Coating</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>MG Chemicals 422C silicone brush-on 55mL, UV indicator, UL 94V-0</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>~$10-15</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>ZWMSSLL 1200pc kit</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Silicone O-Rings</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>~12mm OD x 1mm silicone assortment</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>$35.82</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Brush-on silicone conformal coating. UV indicator for inspection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1" s="11">
+      <c r="A14" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>RTV Silicone Adhesive</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Permatex Clear RTV</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>~$5-8</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>SILICONE not nitrile</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>ePTFE Vent Membrane</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>IP67 adhesive breathable discs</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>~$5-15</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Search "ePTFE waterproof vent adhesive"</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>CONSUMABLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Conformal Coating</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>MG Chemicals 422B silicone spray</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>~$8</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Bonds frame to PCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1" s="11">
+      <c r="A15" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Loctite 222 purple</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>~$15</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>One can = hundreds of units</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>RTV Silicone Adhesive</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Permatex Clear RTV</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>~$10</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Low-strength = removable</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1" s="11">
+      <c r="A16" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Silicone Grease</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Super Lube tube</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>~$8</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Bonds frame to PCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Threadlocker</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Loctite 222 purple</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>~$10</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Low-strength = removable</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Silicone Grease</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Super Lube tube</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>~$6</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Screw sockets + O-ring lube</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>PCB FABRICATION</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="7" t="n">
+    <row r="18" ht="40" customHeight="1" s="11">
+      <c r="A18" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Custom PCBs x5</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>2-layer 0.8mm FR4 ENIG ~16x40mm</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>~$5-10</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Min order 5. Upload Gerbers after KiCad.</t>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Min order 5. Upload Gerbers from Fusion 360.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Amazon/Other Total</t>
         </is>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>~$75-104</t>
         </is>
       </c>
-      <c r="F19" s="9" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="F19" s="4" t="n"/>
+    </row>
+    <row r="21" ht="17" customHeight="1" s="11">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>GRAND TOTAL: DigiKey (~$283) + Amazon (~$75-104) = ~$358-387</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Dev tools (NRF52-DK + PPK2) = $219 one-time. Recurring per-sensor cost = ~$21.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A7:F7"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -1525,299 +1507,295 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" style="11" min="1" max="1"/>
+    <col width="38" customWidth="1" style="11" min="2" max="2"/>
+    <col width="20" customWidth="1" style="11" min="3" max="3"/>
+    <col width="55" customWidth="1" style="11" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="19" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Order Priority Checklist</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Red = order now. Orange = after schematic. Green = anytime.</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>ORDER NOW — Need for firmware dev</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="5" ht="30" customHeight="1" s="11">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>NRF52-DK dev board</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>$52.77 — firmware dev while waiting for PCBs</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+    <row r="6" ht="30" customHeight="1" s="11">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>NRF-PPK2 Power Profiler</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>$166.61 — power optimization</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="7" ht="30" customHeight="1" s="11">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>MDBT42Q-512KV2 x3</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>DigiKey/LCSC</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>$14.85 — Marketplace, backup LCSC</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="8" ht="30" customHeight="1" s="11">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>MS583730BA01-50 x3</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>$33.27 — 6.4k in stock</t>
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>ORDER AFTER KICAD DONE</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+    <row r="11" ht="30" customHeight="1" s="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Custom PCBs x5</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>~$5-10. Need Gerbers. 5-10 day lead.</t>
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>ORDER ANYTIME</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="14" ht="30" customHeight="1" s="11">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>LIS2DH12TR x3 + GRM31CR60J107ME39L x3 + BHSD-1225-SM x3</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>LIS2DH12TR x3 (DigiKey) + GRM31CR60J227ME11L x3 (DigiKey) + no battery holder needed (PCB pad + lid spring)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Add to DigiKey order — $14.49 total</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="15" ht="30" customHeight="1" s="11">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Passives (caps x20 + resistors x20)</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Add to DigiKey order — $0.62 total</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="16" ht="30" customHeight="1" s="11">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>CR1225 batteries x5</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>$3-5</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="17" ht="30" customHeight="1" s="11">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Screws + heat-set inserts kits</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>~$18-27</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="18" ht="30" customHeight="1" s="11">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>O-rings + ePTFE membrane</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Amazon/AliExpress</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>~$10-23</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+    <row r="19" ht="30" customHeight="1" s="11">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Consumables (coat, RTV, Loctite, grease)</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>~$39</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A13:D13"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1829,261 +1807,253 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" style="11" min="1" max="1"/>
+    <col width="20" customWidth="1" style="11" min="2" max="2"/>
+    <col width="15" customWidth="1" style="11" min="3" max="5"/>
+    <col width="10" customWidth="1" style="11" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="19" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Component Verification Matrix</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Voltage OK?</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>I2C Conflict?</t>
         </is>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Fits Enclosure?</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Temp Range?</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Stock?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>MDBT42Q-512KV2</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>1.7-3.6V ✓</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>10.5x15.5x2.2mm ✓</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>-40/+85°C ✓</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>MS5837-30BA</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>1.5-3.6V ✓</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>0x76 ✓</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>3.3x3.3x2.75mm ✓</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>-20/+85°C ⚠</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>&gt;6400</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>LIS2DH12TR</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>1.71-3.6V ✓</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>0x19 ✓</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>2x2x1mm ✓</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>-40/+85°C ✓</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>&gt;77000</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>GRM31CR60J227ME11L</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>6.3V rated ✓</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>3.2x1.6x1.6mm ✓</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>-55/+85°C ✓</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Millions</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>BHSD-1225-SM</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>CR1225 pad + lid spring</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>12mm dia x3mm ✓</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>~12mm pad, fits 16mm board ✓</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>&gt;5800</t>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>N/A (custom)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>CR1225 battery</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>3.0V nom ✓</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>12.5x2.5mm ✓</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>-30/+70°C ✓</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>⚠ MS5837-30BA temp range: sensor functions below -20°C but accuracy not guaranteed. Test during prototyping.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add BeCu spring sheet to BOM for battery lid contacts
C17200 Beryllium Copper Foil 0.1x200x200mm from AliExpress, C$6.22.
Used to cut small leaf springs for enclosure lid battery contacts.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -1082,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="11" min="1" max="1"/>
@@ -1304,39 +1304,41 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BeCu Spring Sheet</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>C17200 Beryllium Copper Foil 0.1x200x200mm, for lid battery spring contacts</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>C$6.22</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Cut small leaf spring per sensor. 200x200mm sheet = lifetime supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1" s="11">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>CONSUMABLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1" s="11">
-      <c r="A13" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Conformal Coating</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>MG Chemicals 422C silicone brush-on 55mL, UV indicator, UL 94V-0</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>$35.82</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Brush-on silicone conformal coating. UV indicator for inspection.</t>
         </is>
       </c>
     </row>
@@ -1346,12 +1348,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>RTV Silicone Adhesive</t>
+          <t>Conformal Coating</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Permatex Clear RTV</t>
+          <t>MG Chemicals 422C silicone brush-on 55mL, UV indicator, UL 94V-0</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1361,12 +1363,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>~$8</t>
+          <t>$35.82</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Bonds frame to PCB</t>
+          <t>Brush-on silicone conformal coating. UV indicator for inspection.</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1378,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Threadlocker</t>
+          <t>RTV Silicone Adhesive</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Loctite 222 purple</t>
+          <t>Permatex Clear RTV</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1391,12 +1393,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>~$10</t>
+          <t>~$8</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Low-strength = removable</t>
+          <t>Bonds frame to PCB</t>
         </is>
       </c>
     </row>
@@ -1406,89 +1408,121 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Loctite 222 purple</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>~$10</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Low-strength = removable</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>Silicone Grease</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Super Lube tube</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>~$6</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Screw sockets + O-ring lube</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="18" ht="40" customHeight="1" s="11">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>PCB FABRICATION</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1" s="11">
-      <c r="A18" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Custom PCBs x5</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>2-layer 0.8mm FR4 ENIG ~16x40mm</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>~$5-10</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Min order 5. Upload Gerbers from Fusion 360.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Amazon/Other Total</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>~$75-104</t>
         </is>
       </c>
-      <c r="F19" s="4" t="n"/>
-    </row>
-    <row r="21" ht="17" customHeight="1" s="11">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="F20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="17" customHeight="1" s="11"/>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>GRAND TOTAL: DigiKey (~$283) + Amazon (~$75-104) = ~$358-387</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Dev tools (NRF52-DK + PPK2) = $219 one-time. Recurring per-sensor cost = ~$21.</t>
         </is>
@@ -1529,7 +1563,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1625,7 +1658,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
@@ -1655,7 +1687,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
BOM: add 150pF NFC caps + 10uH inductor line items, fix PPK2 price, add stencil; document L1 footprint and reverse-battery caveats
- 150pF C0G (GRM1555C1H151JA01D) and 10uH inductor promoted from a
  buried note to real DigiKey line items with verified prices
- L1: no 0402 10uH part meets nRF52832 DC-DC needs; spec 0603
  LQM18DN100M70L (Isat 100mA) overhang-soldered, LDO mode as fallback,
  footprint fix queued for Rev 2 (v2 roadmap)
- PPK2 price corrected to $107.30 (was stale $166.61); totals updated
- Solder paste stencil added (LIS2DH12 LGA-12 needs it)
- Panasonic-only note on CR1225 (cold-weather rating)
- Reverse-battery risk documented; lid polarity marking required
- O-ring size verification note in enclosure README
- Removed stale SMTM1225 battery clip reference from assembly steps

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="11" min="1" max="1"/>
@@ -610,7 +610,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Updated 2026-04-02. All parts verified against design spec + datasheets.</t>
+          <t>Updated 2026-08-13. All parts verified against design spec + PCB netlist (OPENTPMSv1 Rev 1) + datasheets.</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Yageo 1%. I2C pull-ups. 150 min qty on Mouser. ALSO ORDER: 6x 150pF 0402 NFC tuning caps + 3x 10uH 0402 inductors (DC-DC). Add to Mouser order.</t>
+          <t>Yageo 1%. I2C pull-ups. 150 min qty on Mouser.</t>
         </is>
       </c>
     </row>
@@ -968,105 +968,181 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>150pF NFC Tuning Caps (0402)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GRM1555C1H151JA01D</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>$0.10</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>$0.60</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Murata C0G/NP0 50V ±5%. NFC antenna tuning — C5/C6 on PCB. 99k+ in stock. Price verified 2026-08-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1" s="11">
+      <c r="A15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10µH DC-DC Inductor (0603)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>LQM18DN100M70L</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>$0.13</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>$0.39</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Murata shielded multilayer. Isat 100mA, rated 300mA, DCR 1.37Ω max — meets nRF52832 DC-DC requirement (≥50mA). ⚠ 0603 part on 0402 pads (L1): solder with slight overhang. Fallback: leave unpopulated + run LDO mode (skip DCDCEN). Fix footprint to 0603 in Rev 2. 187k+ in stock. Price verified 2026-08-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1" s="11">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>DEV TOOLS (one-time)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="50" customHeight="1" s="11">
-      <c r="A15" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>nRF52-DK Dev Board</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>NRF52-DK</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>$52.77</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>$52.77</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Nordic. Built-in J-Link. Firmware dev before PCBs arrive. 656 in stock.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="50" customHeight="1" s="11">
-      <c r="A16" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Power Profiler Kit II</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>NRF-PPK2</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>$166.61</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>$166.61</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Nordic. nA-level current measurement. 561 in stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>$107.30</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>$107.30</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Nordic. nA-level current measurement. Price verified 2026-08-13: $107.30 DigiKey, 1116 in stock (was listed $166.61 — stale).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1" s="11">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>DigiKey Order Total</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>~$282.76</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="n"/>
-    </row>
-    <row r="19" ht="35" customHeight="1" s="11">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>VERIFIED: All voltages compatible with CR1225 (3.0V). No I2C address conflicts (0x76 + 0x19). All components fit enclosure height budget (≤3.0mm). All in stock.</t>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>~$217.81</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>VERIFIED: All voltages compatible with CR1225 (3.0V). No I2C address conflicts (0x76 + 0x19). All components fit enclosure height budget (≤3.0mm) except L1 caveat (0603 on 0402 pads, 0.8mm tall — fits). All in stock. 150pF caps + 10µH inductor promoted to line items 2026-08-13 (were note-only).</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="11" min="1" max="1"/>
@@ -1107,6 +1183,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1172,7 +1249,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>3 installed + 2 spares</t>
+          <t>3 installed + 2 spares. Panasonic brand specifically — the −30°C cold-weather spec depends on it. Avoid generic/no-name cells.</t>
         </is>
       </c>
     </row>
@@ -1495,38 +1572,70 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Min order 5. Upload Gerbers from Fusion 360.</t>
+          <t>DONE — Rev 1 boards received from PCBWay (sponsored). Line kept for Rev 2 reference.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Solder Paste Stencil</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Stainless stencil from OPENTPMSv1 solderpaste gerber</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>JLCPCB/PCBWay</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>~$10-15</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Order standalone (boards already fabbed). Needed for LIS2DH12 2x2mm LGA-12 — hand paste without stencil is unreliable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1" s="11">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Amazon/Other Total</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>~$75-104</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="17" customHeight="1" s="11"/>
-    <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL: DigiKey (~$283) + Amazon (~$75-104) = ~$358-387</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>~$85-119</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n"/>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL: DigiKey (~$218) + Amazon (~$85-119) = ~$303-337</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Dev tools (NRF52-DK + PPK2) = $219 one-time. Recurring per-sensor cost = ~$21.</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Dev tools (NRF52-DK + PPK2) = $160 one-time. Recurring per-sensor cost = ~$19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1610,7 +1719,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>$166.61 — power optimization</t>
+          <t>$107.30 — power optimization</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1792,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>~$5-10. Need Gerbers. 5-10 day lead.</t>
+          <t>DONE — Rev 1 received from PCBWay (sponsored). NEW: order paste stencil ~$10-15 (standalone).</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1833,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Passives (caps x20 + resistors x20)</t>
+          <t>Passives (100nF x20, 4.7k x10, 100Ω x10, 150pF x6, 10µH LQM18DN100M70L x3)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1734,7 +1843,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Add to DigiKey order — $0.62 total</t>
+          <t>Add to DigiKey order — $1.61 total</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="11" min="1" max="1"/>
@@ -2078,9 +2187,80 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GRM1555C1H151JA01D (150pF C0G)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>50V rated ✓</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0402, 0.6mm ✓</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-55/+125°C ✓</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>&gt;99k</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LQM18DN100M70L (10µH)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0603 on 0402 pads ⚠ overhang-solder; 0.8mm tall ✓</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-55/+125°C ✓</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>&gt;187k</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>⚠ MS5837-30BA temp range: sensor functions below -20°C but accuracy not guaranteed. Test during prototyping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>⚠ L1 footprint is 0402 on Rev 1 PCB but no suitable 0402 10µH power inductor exists (typical Isat 5-30mA &lt; nRF52832 DC-DC need). Plan: overhang-solder the 0603 LQM18DN100M70L; if it fails, run LDO mode (don't set DCDCEN) and fix footprint in Rev 2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM: refresh MDBT42Q sourcing — LCSC OOS, Mouser BO; Amazon/TME/Marketplace options + P-variant drop-in
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Raytac. 1.7-3.6V. Marketplace item — may need manual search. Backup: LCSC $5.96.</t>
+          <t>Raytac. 1.7-3.6V. Current version (no successor — nRF52832 is the ANT++BLE chip). Sourcing verified 2026-08-13: DigiKey Marketplace $4.95 x33 (+$25 flat marketplace ship, ~14 days; 3pcs lands ~$40); Raytac official Amazon store 3-pc pack (check price, usually cheapest landed); TME $6.50/1 (verify stock); LCSC OOS; Mouser BO. Drop-in alternate if chip-antenna dries up: MDBT42Q-P512KV2 (PCB antenna, same footprint/pinout) — $4.80 x50 DigiKey Marketplace.</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1619,7 +1618,6 @@
       </c>
       <c r="F21" s="4" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
BOM: switch CR1225 to Renata via Mouser (-40C rating; Amazon Panasonic listings are BR chemistry)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -1183,6 +1183,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1233,22 +1234,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Panasonic CR1225 x5</t>
+          <t>Renata CR1225 x5-6 (614-CR1225.SC or .IB)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>$3-5</t>
+          <t>~$5-10</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>3 installed + 2 spares. Panasonic brand specifically — the −30°C cold-weather spec depends on it. Avoid generic/no-name cells.</t>
+          <t>SWITCHED 2026-08-13: Renata (Mouser) instead of Panasonic (Amazon). Renata CR series rated -40/+85C (beats Panasonic -30/+70). Amazon Panasonic listings are BR1225 — wrong chemistry (high IR, weak pulse). Rides free in the Mouser PPK2 order. Generic Amazon cells OK as bench spares only.</t>
         </is>
       </c>
     </row>
@@ -1618,6 +1619,7 @@
       </c>
       <c r="F21" s="4" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Docs: PAO grease not silicone on silicone o-rings; Loctite 222 vs blue rationale; coating sourced via Canadian MG distributors
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -1435,7 +1435,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Electro Sonic / ABRA (Canada)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Brush-on silicone conformal coating. UV indicator for inspection.</t>
+          <t>DigiKey/Mouser will not ship chemicals to Canada; Amazon.ca scalped ($79.89). Order 422C-55ML from e-sonic.com (authorized MG distributor) or abra-electronics.com.</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Low-strength = removable</t>
+          <t>ON HAND: blue 242/243 — bench use only, sparingly. Buy 222 purple before ride-test builds: blue break-away torque can round M1.4 hex or spin heat-set inserts in ABS. No threadlocker during bench prototyping.</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Silicone Grease</t>
+          <t>Grease (screw sockets + o-rings)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Super Lube tube</t>
+          <t>Super Lube Multi-Purpose (PAO+PTFE) — ON HAND</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1530,12 +1530,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>~$6</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Screw sockets + O-ring lube</t>
+          <t>SPEC FIX 2026-08-13: do NOT use silicone grease — silicone oil swells silicone o-rings. PAO-based Super Lube MP is silicone-elastomer-safe and covers both socket-fill and o-ring lube.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM: add PROD To-Buy sheet (Loctite 222, 422C coating, SAC305 option) so deferred items aren't forgotten
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amazon &amp; Other" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Priority" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROD To-Buy" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1445,7 +1446,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>DigiKey/Mouser will not ship chemicals to Canada; Amazon.ca scalped ($79.89). Order 422C-55ML from e-sonic.com (authorized MG distributor) or abra-electronics.com.</t>
+          <t>Prototypes: thin coat of the Permatex RTV (same cart) on exposed strip. Real 422C deferred → see PROD To-Buy sheet.</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1506,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>ON HAND: blue 242/243 — bench use only, sparingly. Buy 222 purple before ride-test builds: blue break-away torque can round M1.4 hex or spin heat-set inserts in ABS. No threadlocker during bench prototyping.</t>
+          <t>Bench: NO threadlocker. Blue on hand for emergencies. Loctite 222 → see PROD To-Buy sheet.</t>
         </is>
       </c>
     </row>
@@ -2267,4 +2268,146 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" style="11" min="2" max="2"/>
+    <col width="100" customWidth="1" style="11" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>PROD BUILDS — BUY BEFORE RIDE-TEST / FINAL ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Deferred on purpose during bench prototyping (2026-08-13). Do NOT ship a ride unit without these.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Est. Price</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Why deferred / why required</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Loctite 222 (PURPLE, low-strength)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>~$10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Bench builds use NO threadlocker (constant disassembly). On-hand blue 242/243 is bench-emergency only — medium-strength break-away can round the M1.4 1.3mm hex or spin heat-set inserts out of ABS. Ride units need 222: vibration environment + must stay serviceable for battery swaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MG Chemicals 422C-55ML conformal coating</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Electro Sonic (e-sonic.com) or ABRA / RP Electronics Burnaby / Lee's Vancouver</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>~$30-40</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Prototypes use a THIN coat of Permatex clear RTV on the exposed PCB strip instead (validate in submersion + sealant test). 422C for final builds: proper 50um film, UV inspection indicator, keeps rim-seal seating area thin. DigiKey/Mouser won't ship chemicals to Canada; Amazon.ca scalped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SAC305 solder paste (standard-temp)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Amazon/DigiKey</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>~$15-20</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OPTIONAL BUT RECOMMENDED: bench builds use Chip Quik Sn42/Bi57 low-temp (easy on hot plate) but bismuth joints are brittle under sustained vibration. Consider reflowing ride units in SAC305, or ride-test a low-temp board first and decide on evidence.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mounting clarified: Outrider-style stem clamp needs removable-seal tubeless valves; Rev 1 valve hole 6.0mm must be enlarged to 6.7mm
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpenTPMS_BOM.xlsx
+++ b/docs/OpenTPMS_BOM.xlsx
@@ -1159,7 +1159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="11" min="1" max="1"/>
@@ -1414,84 +1414,86 @@
       </c>
     </row>
     <row r="13" ht="40" customHeight="1" s="11">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tubeless Valves (removable rim seal)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CushCore / Peaty's MK2 / Reserve Fillmore — cone must slide off the stem (NOT Stan's or DT Swiss)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>LBS / check parts bin</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>~C$30-40/pair</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Sensor mounts Outrider-style: valve head clamps PCB above the cone; cone seals rim as stock. Rev 1 PCB hole must be hand-enlarged 6.0→6.7mm first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1" s="11">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>CONSUMABLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1" s="11">
-      <c r="A14" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Conformal Coating</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>MG Chemicals 422C silicone brush-on 55mL, UV indicator, UL 94V-0</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Electro Sonic / ABRA (Canada)</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>$35.82</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Prototypes: thin coat of the Permatex RTV (same cart) on exposed strip. Real 422C deferred → see PROD To-Buy sheet.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1" s="11">
       <c r="A15" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>RTV Silicone Adhesive</t>
+          <t>Conformal Coating</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Permatex Clear RTV</t>
+          <t>MG Chemicals 422C silicone brush-on 55mL, UV indicator, UL 94V-0</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Electro Sonic / ABRA (Canada)</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>~$8</t>
+          <t>$35.82</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Bonds frame to PCB</t>
+          <t>Prototypes: thin coat of the Permatex RTV (same cart) on exposed strip. Real 422C deferred → see PROD To-Buy sheet.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1" s="11">
       <c r="A16" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Threadlocker</t>
+          <t>RTV Silicone Adhesive</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Loctite 222 purple</t>
+          <t>Permatex Clear RTV</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1501,142 +1503,172 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>~$10</t>
+          <t>~$8</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Bench: NO threadlocker. Blue on hand for emergencies. Loctite 222 → see PROD To-Buy sheet.</t>
+          <t>Bonds frame to PCB</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Loctite 222 purple</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>~$10</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Bench: NO threadlocker. Blue on hand for emergencies. Loctite 222 → see PROD To-Buy sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1" s="11">
+      <c r="A18" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Grease (screw sockets + o-rings)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Super Lube Multi-Purpose (PAO+PTFE) — ON HAND</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>SPEC FIX 2026-08-13: do NOT use silicone grease — silicone oil swells silicone o-rings. PAO-based Super Lube MP is silicone-elastomer-safe and covers both socket-fill and o-ring lube.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1" s="11">
-      <c r="A18" s="17" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>PCB FABRICATION</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
+    <row r="20">
+      <c r="A20" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Custom PCBs x5</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>2-layer 0.8mm FR4 ENIG ~16x40mm</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>~$5-10</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>DONE — Rev 1 boards received from PCBWay (sponsored). Line kept for Rev 2 reference.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="n">
+    <row r="21" ht="17" customHeight="1" s="11">
+      <c r="A21" t="n">
         <v>12</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Solder Paste Stencil</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Stainless stencil from OPENTPMSv1 solderpaste gerber</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>JLCPCB/PCBWay</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>~$10-15</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Order standalone (boards already fabbed). Needed for LIS2DH12 2x2mm LGA-12 — hand paste without stencil is unreliable.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="17" customHeight="1" s="11">
-      <c r="A21" s="14" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Amazon/Other Total</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>~$85-119</t>
         </is>
       </c>
-      <c r="F21" s="4" t="n"/>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="F22" s="4" t="n"/>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>GRAND TOTAL: DigiKey (~$218) + Amazon (~$85-119) = ~$303-337</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Dev tools (NRF52-DK + PPK2) = $160 one-time. Recurring per-sensor cost = ~$19.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="18" t="n"/>
+    <row r="26">
+      <c r="A26" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2289,10 +2321,6 @@
           <t>PROD BUILDS — BUY BEFORE RIDE-TEST / FINAL ASSEMBLY</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2300,10 +2328,6 @@
           <t>Deferred on purpose during bench prototyping (2026-08-13). Do NOT ship a ride unit without these.</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>